<commit_message>
Dash Hedge IPCA - 2026-02-27
</commit_message>
<xml_diff>
--- a/Dados/Ativos_Sem_Codigo.xlsx
+++ b/Dados/Ativos_Sem_Codigo.xlsx
@@ -1,40 +1,99 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="17">
+  <si>
+    <t>Sub Classe</t>
+  </si>
+  <si>
+    <t>Ativo</t>
+  </si>
+  <si>
+    <t>Vencimento_final</t>
+  </si>
+  <si>
+    <t>Fundo</t>
+  </si>
+  <si>
+    <t>ISIN</t>
+  </si>
+  <si>
+    <t>COD_XP</t>
+  </si>
+  <si>
+    <t>LFSN</t>
+  </si>
+  <si>
+    <t>Letra Financeira</t>
+  </si>
+  <si>
+    <t>LFSN1800D4W</t>
+  </si>
+  <si>
+    <t>LFSN1800DS5</t>
+  </si>
+  <si>
+    <t>LFSN19001BC</t>
+  </si>
+  <si>
+    <t>LFSN1800DG1</t>
+  </si>
+  <si>
+    <t>LF002400KC0</t>
+  </si>
+  <si>
+    <t>BH INFRA</t>
+  </si>
+  <si>
+    <t>BORDEAUX INFRA</t>
+  </si>
+  <si>
+    <t>CARMEL INFRA</t>
+  </si>
+  <si>
+    <t>BMG SEG</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
   <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -49,94 +108,36 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
 </file>
 
@@ -424,91 +425,115 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Sub Classe</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Vencimento_final</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Fundo</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>ISIN</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>COD_XP</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>CDB</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>CDB424EERW3</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>46146</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>BBRASIL FIM</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>CDB</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>CDB3239C4TL</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>46223</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>BBRASIL FIM</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
+    <row r="1" spans="1:6">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="2">
+        <v>46181</v>
+      </c>
+      <c r="D2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="2">
+        <v>46251</v>
+      </c>
+      <c r="D3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="2">
+        <v>46251</v>
+      </c>
+      <c r="D4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="2">
+        <v>46486</v>
+      </c>
+      <c r="D5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="2">
+        <v>46237</v>
+      </c>
+      <c r="D6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="2">
+        <v>46234</v>
+      </c>
+      <c r="D7" t="s">
+        <v>16</v>
+      </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Dash CDI - 19/03/2026
</commit_message>
<xml_diff>
--- a/Dados/Ativos_Sem_Codigo.xlsx
+++ b/Dados/Ativos_Sem_Codigo.xlsx
@@ -1,99 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr defaultThemeVersion="124226"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="17">
-  <si>
-    <t>Sub Classe</t>
-  </si>
-  <si>
-    <t>Ativo</t>
-  </si>
-  <si>
-    <t>Vencimento_final</t>
-  </si>
-  <si>
-    <t>Fundo</t>
-  </si>
-  <si>
-    <t>ISIN</t>
-  </si>
-  <si>
-    <t>COD_XP</t>
-  </si>
-  <si>
-    <t>LFSN</t>
-  </si>
-  <si>
-    <t>Letra Financeira</t>
-  </si>
-  <si>
-    <t>LFSN1800D4W</t>
-  </si>
-  <si>
-    <t>LFSN1800DS5</t>
-  </si>
-  <si>
-    <t>LFSN19001BC</t>
-  </si>
-  <si>
-    <t>LFSN1800DG1</t>
-  </si>
-  <si>
-    <t>LF002400KC0</t>
-  </si>
-  <si>
-    <t>BH INFRA</t>
-  </si>
-  <si>
-    <t>BORDEAUX INFRA</t>
-  </si>
-  <si>
-    <t>CARMEL INFRA</t>
-  </si>
-  <si>
-    <t>BMG SEG</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
   <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -108,36 +49,94 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -425,115 +424,91 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Sub Classe</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Vencimento_final</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Fundo</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ISIN</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>COD_XP</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:6">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="2">
-        <v>46181</v>
-      </c>
-      <c r="D2" t="s">
-        <v>13</v>
-      </c>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>LFSN</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>LFSN19009YU</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>46199</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>CARMEL INFRA</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
     </row>
-    <row r="3" spans="1:6">
-      <c r="A3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="2">
-        <v>46251</v>
-      </c>
-      <c r="D3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" s="2">
-        <v>46251</v>
-      </c>
-      <c r="D4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
-      <c r="A5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" s="2">
-        <v>46486</v>
-      </c>
-      <c r="D5" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
-      <c r="A6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" s="2">
-        <v>46237</v>
-      </c>
-      <c r="D6" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6">
-      <c r="A7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" s="2">
-        <v>46234</v>
-      </c>
-      <c r="D7" t="s">
-        <v>16</v>
-      </c>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CDB</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>CDB3251WXH0</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>46454</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>CARMEL INFRA</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Dash CDI - 19/05/2026
</commit_message>
<xml_diff>
--- a/Dados/Ativos_Sem_Codigo.xlsx
+++ b/Dados/Ativos_Sem_Codigo.xlsx
@@ -1,93 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\Asset Management\Equipe\Lívia\HedgeCDI\Projeto-Hedge-CDI\Dados\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2DF202A-AEE3-47C8-BEFC-6DFEF9524387}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
-  <si>
-    <t>Sub Classe</t>
-  </si>
-  <si>
-    <t>Ativo</t>
-  </si>
-  <si>
-    <t>Vencimento_final</t>
-  </si>
-  <si>
-    <t>Fundo</t>
-  </si>
-  <si>
-    <t>ISIN</t>
-  </si>
-  <si>
-    <t>COD_XP</t>
-  </si>
-  <si>
-    <t>LFSN</t>
-  </si>
-  <si>
-    <t>LFSN1800D4W</t>
-  </si>
-  <si>
-    <t>BH INFRA</t>
-  </si>
-  <si>
-    <t>BRBSAFLNND73</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -102,44 +49,94 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -427,54 +424,111 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="4.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.140625" bestFit="1" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Sub Classe</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Vencimento_final</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Fundo</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ISIN</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>COD_XP</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="2">
-        <v>46240</v>
-      </c>
-      <c r="D2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" t="s">
-        <v>9</v>
-      </c>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>LFSN</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>LFSN1800D4W</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>CARMEL INFRA</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>LFSN</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>LFSN19001BH</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>46486</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>FIRF GERAES</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>LFSN</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>LFSN1900971</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>46195</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>CARMEL INFRA</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Dash DI - 2026-05-29
</commit_message>
<xml_diff>
--- a/Dados/Ativos_Sem_Codigo.xlsx
+++ b/Dados/Ativos_Sem_Codigo.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -476,7 +476,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46181</v>
+        <v>46240</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -485,50 +485,6 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>LFSN</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>LFSN19001BH</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>46486</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>FIRF GERAES</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>LFSN</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>LFSN1900971</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>46195</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>CARMEL INFRA</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Dash DI - 12/08/2026
</commit_message>
<xml_diff>
--- a/Dados/Ativos_Sem_Codigo.xlsx
+++ b/Dados/Ativos_Sem_Codigo.xlsx
@@ -37,10 +37,10 @@
     <t>CDB</t>
   </si>
   <si>
-    <t>CDB3239C4TL</t>
-  </si>
-  <si>
-    <t>FIRF GERAES</t>
+    <t>CDB3251WXH0</t>
+  </si>
+  <si>
+    <t>REAL FIM</t>
   </si>
 </sst>
 </file>
@@ -433,7 +433,7 @@
         <v>7</v>
       </c>
       <c r="C2" s="2">
-        <v>46223</v>
+        <v>46454</v>
       </c>
       <c r="D2" t="s">
         <v>8</v>

</xml_diff>